<commit_message>
Introduction configuration de connexion symétrique
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS SFS01/Cas SFS01b.xlsx
+++ b/VALIDATION/CAS SFS01/Cas SFS01b.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS SFS01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB3E4D0-E68D-4895-984B-569E578E9F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDB7C02D-F2F5-4DD3-AE1B-28C9034CAF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -961,7 +961,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1208,9 +1208,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2457,7 +2454,7 @@
       </c>
       <c r="J36" s="52">
         <f>MEd_U1/'Section élastique'!P54</f>
-        <v>1.195924743168943</v>
+        <v>1.1924811797297832</v>
       </c>
       <c r="M36" s="41" t="s">
         <v>95</v>
@@ -3481,10 +3478,10 @@
       <c r="C17" t="s">
         <v>139</v>
       </c>
-      <c r="L17" s="102" t="s">
+      <c r="L17" s="101" t="s">
         <v>92</v>
       </c>
-      <c r="M17" s="102" t="s">
+      <c r="M17" s="101" t="s">
         <v>140</v>
       </c>
     </row>
@@ -3519,12 +3516,12 @@
         <v>163</v>
       </c>
       <c r="L19" s="54">
-        <f>qELU*L18/1000*1000</f>
-        <v>2174.0024035110209</v>
+        <f>qELU*L18/1000*1000/2</f>
+        <v>1087.0012017555105</v>
       </c>
       <c r="M19" s="54">
-        <f>qELU*M18/1000*1000</f>
-        <v>2945.3384562767305</v>
+        <f>qELU*M18/1000*1000/2</f>
+        <v>1472.6692281383653</v>
       </c>
     </row>
     <row r="20" spans="3:18" x14ac:dyDescent="0.25">
@@ -3551,7 +3548,7 @@
       </c>
     </row>
     <row r="21" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="K21" s="101" t="s">
+      <c r="K21" s="3" t="s">
         <v>165</v>
       </c>
       <c r="L21" s="5">
@@ -3595,11 +3592,11 @@
       </c>
       <c r="L23" s="53">
         <f>L19/L22</f>
-        <v>0.20557942349986014</v>
+        <v>0.10278971174993007</v>
       </c>
       <c r="M23" s="53">
         <f>M19/M22</f>
-        <v>0.54735588842224092</v>
+        <v>0.27367794421112046</v>
       </c>
     </row>
     <row r="24" spans="3:18" x14ac:dyDescent="0.25">
@@ -3618,11 +3615,11 @@
       </c>
       <c r="L24" s="53">
         <f>(L23-SQRT(L23^2-16*L23+16))/(2*(L23-2))</f>
-        <v>0.93778286744617434</v>
+        <v>0.97180891665940616</v>
       </c>
       <c r="M24" s="53">
         <f>(M23-SQRT(M23^2-16*M23+16))/(2*(M23-2))</f>
-        <v>0.75686014898050813</v>
+        <v>0.91126428066996557</v>
       </c>
     </row>
     <row r="25" spans="3:18" x14ac:dyDescent="0.25">
@@ -3766,7 +3763,7 @@
       </c>
       <c r="Q30" s="59">
         <f>O36-O30</f>
-        <v>1787.4064974574924</v>
+        <v>1881.6264228704561</v>
       </c>
       <c r="R30" s="59">
         <f>O30</f>
@@ -3817,7 +3814,7 @@
       </c>
       <c r="Q31" s="59">
         <f>Q30-O31</f>
-        <v>1739.6848532367726</v>
+        <v>1833.9047786497363</v>
       </c>
       <c r="R31" s="59">
         <f>R30+O31</f>
@@ -3868,7 +3865,7 @@
       </c>
       <c r="Q32" s="59">
         <f t="shared" ref="Q32:Q35" si="6">Q31-O32</f>
-        <v>1324.8957532367726</v>
+        <v>1419.1156786497363</v>
       </c>
       <c r="R32" s="59">
         <f t="shared" ref="R32:R35" si="7">R31+O32</f>
@@ -3919,7 +3916,7 @@
       </c>
       <c r="Q33" s="59">
         <f t="shared" si="6"/>
-        <v>1277.1741090160529</v>
+        <v>1371.3940344290165</v>
       </c>
       <c r="R33" s="59">
         <f t="shared" si="7"/>
@@ -3936,11 +3933,11 @@
       </c>
       <c r="N34" s="59">
         <f>FyI/GammaM0*M24</f>
-        <v>177.86213501041942</v>
+        <v>214.14710595744191</v>
       </c>
       <c r="O34" s="59">
         <f t="shared" si="5"/>
-        <v>285.46872669172313</v>
+        <v>343.7061050616943</v>
       </c>
       <c r="P34" s="4">
         <f>Feuil1!Q39</f>
@@ -3948,11 +3945,11 @@
       </c>
       <c r="Q34" s="59">
         <f t="shared" si="6"/>
-        <v>991.70538232432978</v>
+        <v>1027.6879293673223</v>
       </c>
       <c r="R34" s="59">
         <f t="shared" si="7"/>
-        <v>1172.876115133163</v>
+        <v>1231.1134935031341</v>
       </c>
     </row>
     <row r="35" spans="3:21" x14ac:dyDescent="0.25">
@@ -3965,11 +3962,11 @@
       </c>
       <c r="N35" s="75">
         <f>FyPl/GammaM0*L24</f>
-        <v>220.37897384985098</v>
+        <v>228.37509541496044</v>
       </c>
       <c r="O35" s="59">
         <f t="shared" si="5"/>
-        <v>991.70538232432943</v>
+        <v>1027.6879293673221</v>
       </c>
       <c r="P35" s="4">
         <f>Feuil1!Q40</f>
@@ -3981,7 +3978,7 @@
       </c>
       <c r="R35" s="59">
         <f t="shared" si="7"/>
-        <v>2164.5814974574923</v>
+        <v>2258.801422870456</v>
       </c>
     </row>
     <row r="36" spans="3:21" x14ac:dyDescent="0.25">
@@ -3991,7 +3988,7 @@
       </c>
       <c r="O36" s="55">
         <f>SUM(O30:O35)</f>
-        <v>2164.5814974574923</v>
+        <v>2258.801422870456</v>
       </c>
     </row>
     <row r="40" spans="3:21" x14ac:dyDescent="0.25">
@@ -4005,7 +4002,7 @@
       </c>
       <c r="M42" s="52">
         <f>(O36-2*O35)/2/O34</f>
-        <v>0.31732150647184415</v>
+        <v>0.29592951818428925</v>
       </c>
     </row>
     <row r="43" spans="3:21" x14ac:dyDescent="0.25">
@@ -4014,7 +4011,7 @@
       </c>
       <c r="M43" s="53">
         <f>M42*tf</f>
-        <v>3.3953401192487322</v>
+        <v>3.1664458445718946</v>
       </c>
       <c r="N43" t="s">
         <v>2</v>
@@ -4048,11 +4045,11 @@
       </c>
       <c r="O47" s="67">
         <f>N47-$M$43</f>
-        <v>291.25465988075126</v>
+        <v>291.48355415542807</v>
       </c>
       <c r="P47" s="88">
         <f>M47*ABS(O47/1000)</f>
-        <v>109.85397634052237</v>
+        <v>109.9403095385736</v>
       </c>
       <c r="R47" s="59">
         <f>Feuil1!N52</f>
@@ -4085,11 +4082,11 @@
       </c>
       <c r="O48" s="68">
         <f>N48-$M$43</f>
-        <v>282.55414079656504</v>
+        <v>282.78303507124184</v>
       </c>
       <c r="P48" s="90">
         <f t="shared" ref="P48:P53" si="9">M48*ABS(O48/1000)</f>
-        <v>13.483948180184861</v>
+        <v>13.494871391325146</v>
       </c>
       <c r="R48" s="59">
         <f>Feuil1!N53</f>
@@ -4122,11 +4119,11 @@
       </c>
       <c r="O49" s="68">
         <f t="shared" ref="O49:O50" si="11">N49-$M$43</f>
-        <v>146.60465988075126</v>
+        <v>146.83355415542812</v>
       </c>
       <c r="P49" s="90">
         <f t="shared" si="9"/>
-        <v>60.81001492774292</v>
+        <v>60.904957777931294</v>
       </c>
       <c r="R49" s="59">
         <f>Feuil1!N54</f>
@@ -4159,11 +4156,11 @@
       </c>
       <c r="O50" s="68">
         <f t="shared" si="11"/>
-        <v>10.655178964937493</v>
+        <v>10.884073239614331</v>
       </c>
       <c r="P50" s="90">
         <f t="shared" si="9"/>
-        <v>0.50848265967284489</v>
+        <v>0.51940587081313272</v>
       </c>
       <c r="R50" s="59">
         <f>Feuil1!N55</f>
@@ -4188,16 +4185,16 @@
       </c>
       <c r="M51" s="85">
         <f>(1-M42)*O34</f>
-        <v>194.88336028730637</v>
+        <v>241.99332299378841</v>
       </c>
       <c r="N51" s="89"/>
       <c r="O51" s="68">
         <f>(1-M42)*tf/2</f>
-        <v>3.6523299403756333</v>
+        <v>3.7667770777140523</v>
       </c>
       <c r="P51" s="90">
         <f t="shared" si="9"/>
-        <v>0.71177833165834081</v>
+        <v>0.91153490201285514</v>
       </c>
       <c r="R51" s="59">
         <f>Feuil1!N56</f>
@@ -4222,16 +4219,16 @@
       </c>
       <c r="M52" s="85">
         <f>M42*O34</f>
-        <v>90.585366404416732</v>
+        <v>101.71278206790589</v>
       </c>
       <c r="N52" s="89"/>
       <c r="O52" s="68">
         <f>(-M42)*tf/2</f>
-        <v>-1.6976700596243661</v>
+        <v>-1.5832229222859473</v>
       </c>
       <c r="P52" s="90">
         <f t="shared" si="9"/>
-        <v>0.15378406438488121</v>
+        <v>0.16103400805938367</v>
       </c>
       <c r="R52" s="59">
         <f>Feuil1!N57</f>
@@ -4256,7 +4253,7 @@
       </c>
       <c r="M53" s="94">
         <f>O35</f>
-        <v>991.70538232432943</v>
+        <v>1027.6879293673221</v>
       </c>
       <c r="N53" s="91">
         <f>P35</f>
@@ -4264,11 +4261,11 @@
       </c>
       <c r="O53" s="73">
         <f>N53-M43</f>
-        <v>-10.895340119248733</v>
+        <v>-10.666445844571895</v>
       </c>
       <c r="P53" s="92">
         <f t="shared" si="9"/>
-        <v>10.804967438513168</v>
+        <v>10.961777643716768</v>
       </c>
       <c r="R53" s="59">
         <f>Feuil1!N58</f>
@@ -4290,7 +4287,7 @@
     <row r="54" spans="12:21" x14ac:dyDescent="0.25">
       <c r="P54" s="86">
         <f>SUM(P47:P53)</f>
-        <v>196.32695194267936</v>
+        <v>196.89389113243217</v>
       </c>
       <c r="U54" s="86">
         <f>SUM(U47:U53)</f>
@@ -4303,7 +4300,7 @@
       </c>
       <c r="P56" s="76">
         <f>P54</f>
-        <v>196.32695194267936</v>
+        <v>196.89389113243217</v>
       </c>
       <c r="Q56" t="s">
         <v>18</v>
@@ -4327,7 +4324,7 @@
       </c>
       <c r="M58" s="55">
         <f>SUM(M47:M51)</f>
-        <v>1082.2907487287462</v>
+        <v>1129.4007114352282</v>
       </c>
     </row>
     <row r="59" spans="12:21" x14ac:dyDescent="0.25">
@@ -4336,7 +4333,7 @@
       </c>
       <c r="M59" s="55">
         <f>SUM(M52:M53)</f>
-        <v>1082.2907487287462</v>
+        <v>1129.400711435228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>